<commit_message>
CCART v1.1 — Final updates
</commit_message>
<xml_diff>
--- a/data/SID_for_storms.xlsx
+++ b/data/SID_for_storms.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CMIP data\cmip6\Climada\Projects\ccart-india\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7CAD4E1-5FB9-489A-AAD2-892EAEFB1B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55BCF3A-3473-42FB-AD62-F594666F7747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{048AB855-62E3-4884-B9AA-31B480784FD5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{048AB855-62E3-4884-B9AA-31B480784FD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="43">
   <si>
     <t>Storm</t>
   </si>
@@ -47,9 +48,6 @@
     <t>Phailin</t>
   </si>
   <si>
-    <t>2013281N18088</t>
-  </si>
-  <si>
     <t>Hudhud</t>
   </si>
   <si>
@@ -59,25 +57,115 @@
     <t>Fani</t>
   </si>
   <si>
-    <t>2019129N13086</t>
-  </si>
-  <si>
     <t>Amphan</t>
   </si>
   <si>
-    <t>2020135N11088</t>
-  </si>
-  <si>
     <t>Nisarga</t>
   </si>
   <si>
-    <t>2020153N15073</t>
-  </si>
-  <si>
     <t>Tauktae</t>
   </si>
   <si>
-    <t>2021133N15072</t>
+    <t>2020136N10088</t>
+  </si>
+  <si>
+    <t>2019116N02090</t>
+  </si>
+  <si>
+    <t>2020153N13072</t>
+  </si>
+  <si>
+    <t>2013281N12098</t>
+  </si>
+  <si>
+    <t>2021133N10071</t>
+  </si>
+  <si>
+    <t>Sr No.</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>sid</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>basin</t>
+  </si>
+  <si>
+    <t>landfall_state</t>
+  </si>
+  <si>
+    <t>landfall_date</t>
+  </si>
+  <si>
+    <t>dlna_available</t>
+  </si>
+  <si>
+    <t>litpop_ready</t>
+  </si>
+  <si>
+    <t>comments</t>
+  </si>
+  <si>
+    <t>AMPHAN</t>
+  </si>
+  <si>
+    <t>BoB</t>
+  </si>
+  <si>
+    <t>West Bengal</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Landfall near Digha, WB</t>
+  </si>
+  <si>
+    <t>FANI</t>
+  </si>
+  <si>
+    <t>Odisha</t>
+  </si>
+  <si>
+    <t>Landfall near Puri, Odisha</t>
+  </si>
+  <si>
+    <t>NISARGA</t>
+  </si>
+  <si>
+    <t>AS</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>Landfall near Alibag, Maharashtra</t>
+  </si>
+  <si>
+    <t>PHAILIN</t>
+  </si>
+  <si>
+    <t>Landfall near Gopalpur, Odisha</t>
+  </si>
+  <si>
+    <t>TAUKTAE</t>
+  </si>
+  <si>
+    <t>Gujarat</t>
+  </si>
+  <si>
+    <t>Landfall near Diu/Saurashtra coast, Gujarat</t>
+  </si>
+  <si>
+    <t>HUDHUD</t>
   </si>
 </sst>
 </file>
@@ -109,7 +197,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -117,17 +205,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -463,67 +572,306 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15FF17B9-D8A3-412D-BA2D-5FE61C2EF05B}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="B6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="D6">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B6">
+    <sortCondition ref="A1:A6"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9EF900B-20F9-4CF9-A35E-FA009E3916CE}">
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.88671875" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" customWidth="1"/>
+    <col min="9" max="9" width="44.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="B2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="3">
+        <v>2020</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="5">
+        <v>43971</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2019</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="5">
+        <v>43588</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2020</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="5">
+        <v>43985</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2013</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="5">
+        <v>41559</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>13</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="3">
+        <v>2021</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="5">
+        <v>44333</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>